<commit_message>
Provide SQL query handoffs for Alteryx, Tableau, and Fabric
</commit_message>
<xml_diff>
--- a/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
+++ b/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R84a1645f86434ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R802d192dc6134e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="R5c42aa9bed694d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R7d2db8472fab4f20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R4bad28bbb2a44622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R64e3f075cf704573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="Rb2745ead1e02482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="R0fd3570325fa4727"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="Rffcefece92db4af4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R6c63fb1ac3c54da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="R000f124c61d14762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R36b4b8efefaf40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="Rb4146c87a0824024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R7667b00ce4b44ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R24e8e0a5fa244692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="R475635fff4c7467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="Rdc19d97cfb6f403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R35e06569631d4547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R02d97914bffd4fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="Rdfd902765592404b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R306371199fef4693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ff78ae54c4147ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R746ebc82870e40ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R695faf2619634fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="R4a4d6630eb8a4967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="R32fc44687fd641ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R2794a9d89628442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="Re0c316331b194d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R21201718dbd34235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="Re1dc4cb9718f44d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R02803f40f78248bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R27ef375b836d411c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Re42b7c9b960043d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="Raa76edd8102b4f9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -894,7 +894,7 @@
         <x:v>Tableau reference</x:v>
       </x:c>
       <x:c r="B20" s="4" t="str">
-        <x:v>Use the repository mapping in Tableau_Output. Verify installed PostgreSQL columns and joins.</x:v>
+        <x:v>Use the repository mapping in Tableau_Output. Run tableau-postgresql-selects.sql. Verify installed PostgreSQL columns and joins.</x:v>
       </x:c>
       <x:c r="C20" s="4" t="str">
         <x:v>Tableau 2026.2</x:v>
@@ -908,27 +908,27 @@
         <x:v>Power BI reference</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>Use the scanner-output mapping in PowerBI_Output. Product release labels are not identity keys.</x:v>
+        <x:v>Use fabric-inventory.sql for landed Fabric inventory. PowerBI_Output distinguishes its coverage from the richer, existing JSON-export alternative. See fabric-query-mapping.md.</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
         <x:v>Power BI / Fabric</x:v>
       </x:c>
       <x:c r="D21" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="47.25" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="36" customHeight="1">
       <x:c r="A22" s="4" t="str">
         <x:v>Alteryx reference</x:v>
       </x:c>
       <x:c r="B22" s="4" t="str">
-        <x:v>Use MongoDB backend mappings in Alteryx_Output. This profile does not use the Alteryx API.</x:v>
+        <x:v>Run alteryx-sqlserver.sql against SQL Server copies through the documented adapter views. Alteryx_Output uses the linked 2025.1 fields; validate them against your 2025.2 export.</x:v>
       </x:c>
       <x:c r="C22" s="4" t="str">
-        <x:v>Alteryx 2025.2</x:v>
+        <x:v>Alteryx 2025.2 SQL export</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/alteryx-sqlserver-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
@@ -946,7 +946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R673e269a28264483"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37cb9a51087c417a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1020,7 +1020,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54bc222c8287438b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re348627782404da5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1112,7 +1112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R668f394839384cdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref01c47526934f4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1204,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83a11c0527bb4ce5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7a5777105a948f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1278,7 +1278,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b33fe09cb854a73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169aecea494e415e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1397,7 +1397,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refdc4443bbd945d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbccb69c61b1c4f44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3364,7 +3364,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf28c72b741bf4724"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e780e0296d4a40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3782,7 +3782,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="F18" s="4" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -3791,7 +3791,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H18" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
@@ -3808,16 +3808,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>workspaces[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceId. Existing scan export: workspaces[].id</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>Preserve exact source text. Scope comes from Run_Context.</x:v>
+        <x:v>Fabric inventory: Preserve the native workspace ID as text. Existing scan export: Preserve exact source text. Scope comes from Run_Context.</x:v>
       </x:c>
       <x:c r="G19" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H19" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
@@ -3834,16 +3834,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
-        <x:v>Source entity kind</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceType. Existing scan export: Source entity kind</x:v>
       </x:c>
       <x:c r="F20" s="4" t="str">
-        <x:v>Use workspaces[].type, commonly Workspace or PersonalGroup.</x:v>
+        <x:v>Fabric inventory: Use the validated native type. Missing type stops extraction. Existing scan export: Use workspaces[].type, commonly Workspace or PersonalGroup.</x:v>
       </x:c>
       <x:c r="G20" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H20" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
@@ -3860,16 +3860,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
-        <x:v>workspaces[].name</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceName. Existing scan export: workspaces[].name</x:v>
       </x:c>
       <x:c r="F21" s="17" t="str">
-        <x:v>Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
+        <x:v>Fabric inventory: Use the observed name; never use it as a key. Existing scan export: Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
       </x:c>
       <x:c r="G21" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="36" customHeight="1">
@@ -3883,19 +3883,19 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
-        <x:v>workspaces[].state</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: workspaces[].state</x:v>
       </x:c>
       <x:c r="F22" s="4" t="str">
-        <x:v>Preserve the native state; never infer account status.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Preserve the native state; never infer account status.</x:v>
       </x:c>
       <x:c r="G22" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H22" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
@@ -3912,7 +3912,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E23" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="F23" s="17" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -3921,10 +3921,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H23" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="47.25" customHeight="1">
       <x:c r="A24" s="4" t="str">
         <x:v>Assets</x:v>
       </x:c>
@@ -3938,16 +3938,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>workspaces[].reports[].id or datasets[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemId. Existing scan export: workspaces[].reports[].id or datasets[].id</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
-        <x:v>Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
+        <x:v>Fabric inventory: Preserve the native item ID as text. Existing scan export: Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
       </x:c>
       <x:c r="G24" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H24" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
@@ -3964,16 +3964,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E25" s="17" t="str">
-        <x:v>Source object namespace</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemType. Existing scan export: Source object namespace</x:v>
       </x:c>
       <x:c r="F25" s="17" t="str">
-        <x:v>Report or Dataset, matching the source array.</x:v>
+        <x:v>Fabric inventory: Report stays Report. SemanticModel, Semantic model, and Dataset map to Dataset. Existing scan export: Report or Dataset, matching the source array.</x:v>
       </x:c>
       <x:c r="G25" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H25" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
@@ -3990,16 +3990,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>reports[].name or datasets[].name</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemName. Existing scan export: reports[].name or datasets[].name</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
-        <x:v>If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
+        <x:v>Fabric inventory: Use the observed item name. Existing scan export: If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
       </x:c>
       <x:c r="G26" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H26" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="36" customHeight="1">
@@ -4013,19 +4013,19 @@
         <x:v>nvarchar(100)</x:v>
       </x:c>
       <x:c r="D27" s="17" t="str">
-        <x:v>Leave NULL</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E27" s="17" t="str">
-        <x:v>No native revision in the baseline scan fields</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: No native revision in the baseline scan fields</x:v>
       </x:c>
       <x:c r="F27" s="17" t="str">
-        <x:v>Do not synthesize a version from modified time.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Do not synthesize a version from modified time.</x:v>
       </x:c>
       <x:c r="G27" s="17" t="str">
-        <x:v>Always NULL for baseline scan projection.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: Always NULL for baseline scan projection.</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
@@ -4039,19 +4039,19 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>Leave NULL</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
-        <x:v>Not projected by baseline inventory</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: Not projected by baseline inventory</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>Inventory presence is recorded by the observation itself.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Inventory presence is recorded by the observation itself.</x:v>
       </x:c>
       <x:c r="G28" s="4" t="str">
-        <x:v>Always NULL unless an authoritative lifecycle field is separately approved.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: Always NULL unless an authoritative lifecycle field is separately approved.</x:v>
       </x:c>
       <x:c r="H28" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="36" customHeight="1">
@@ -4068,7 +4068,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E29" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="F29" s="17" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -4077,7 +4077,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="36" customHeight="1">
@@ -4094,16 +4094,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
-        <x:v>Parent workspaces[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceId. Existing scan export: Parent workspaces[].id</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
-        <x:v>Resolve exact ID in this delivery scope.</x:v>
+        <x:v>Fabric inventory: Preserve the native workspace ID. Existing scan export: Resolve exact ID in this delivery scope.</x:v>
       </x:c>
       <x:c r="G30" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H30" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="36" customHeight="1">
@@ -4120,16 +4120,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>Nested reports[].id / datasets[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemId. Existing scan export: Nested reports[].id / datasets[].id</x:v>
       </x:c>
       <x:c r="F31" s="17" t="str">
-        <x:v>Preserve unmatched IDs as unresolved relationships.</x:v>
+        <x:v>Fabric inventory: Preserve the native item ID. Existing scan export: Preserve unmatched IDs as unresolved relationships.</x:v>
       </x:c>
       <x:c r="G31" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="36" customHeight="1">
@@ -4146,16 +4146,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemType. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="F32" s="4" t="str">
-        <x:v>Report / Dataset</x:v>
+        <x:v>Fabric inventory: Use Report or Dataset with the same type mapping as Assets. Existing scan export: Report / Dataset</x:v>
       </x:c>
       <x:c r="G32" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H32" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
@@ -4172,19 +4172,19 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E33" s="17" t="str">
-        <x:v>Query relationship label</x:v>
+        <x:v>Fabric inventory: Direct source containment (query constant). Existing scan export: Query relationship label</x:v>
       </x:c>
       <x:c r="F33" s="17" t="str">
-        <x:v>ContainedIn; observed membership never assigns business ownership.</x:v>
+        <x:v>Fabric inventory: Use ContainedIn. This is membership, not lineage. Existing scan export: ContainedIn; observed membership never assigns business ownership.</x:v>
       </x:c>
       <x:c r="G33" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="47.25" customHeight="1">
       <x:c r="A34" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4195,22 +4195,22 @@
         <x:v>uniqueidentifier</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="F34" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="G34" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H34" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="47.25" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4221,22 +4221,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D35" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E35" s="17" t="str">
-        <x:v>datasourceInstances[].datasourceId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceId</x:v>
       </x:c>
       <x:c r="F35" s="17" t="str">
-        <x:v>Exact native datasource ID. Do not hash connection secrets or invent a name-based ID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Exact native datasource ID. Do not hash connection secrets or invent a name-based ID.</x:v>
       </x:c>
       <x:c r="G35" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="47.25" customHeight="1">
       <x:c r="A36" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4247,22 +4247,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
-        <x:v>datasourceInstances[].datasourceType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceType</x:v>
       </x:c>
       <x:c r="F36" s="4" t="str">
-        <x:v>Optional readable technical label. No business meaning is inferred.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Optional readable technical label. No business meaning is inferred.</x:v>
       </x:c>
       <x:c r="G36" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H36" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="47.25" customHeight="1">
       <x:c r="A37" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4273,22 +4273,22 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D37" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E37" s="17" t="str">
-        <x:v>datasourceInstances[].datasourceType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceType</x:v>
       </x:c>
       <x:c r="F37" s="17" t="str">
-        <x:v>Map Oracle to Oracle, Sql to SQL Server; preserve other known types. Undefined only when technology is unavailable.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Map Oracle to Oracle, Sql to SQL Server; preserve other known types. Undefined only when technology is unavailable.</x:v>
       </x:c>
       <x:c r="G37" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="47.25" customHeight="1">
       <x:c r="A38" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4299,22 +4299,22 @@
         <x:v>bit</x:v>
       </x:c>
       <x:c r="D38" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E38" s="4" t="str">
-        <x:v>Not supplied by scan datasource instance</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by scan datasource instance</x:v>
       </x:c>
       <x:c r="F38" s="4" t="str">
-        <x:v>NULL. Report/model storage mode must not be inferred from datasource type.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL. Report/model storage mode must not be inferred from datasource type.</x:v>
       </x:c>
       <x:c r="G38" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H38" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="47.25" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4325,22 +4325,22 @@
         <x:v>nvarchar(255)</x:v>
       </x:c>
       <x:c r="D39" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>datasourceInstances[].connectionDetails.server</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].connectionDetails.server</x:v>
       </x:c>
       <x:c r="F39" s="17" t="str">
-        <x:v>Sanitized host only. No URL tokens or credentials.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Sanitized host only. No URL tokens or credentials.</x:v>
       </x:c>
       <x:c r="G39" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H39" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="47.25" customHeight="1">
       <x:c r="A40" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4351,22 +4351,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>datasourceInstances[].connectionDetails.database</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].connectionDetails.database</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
-        <x:v>Database name when present.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Database name when present.</x:v>
       </x:c>
       <x:c r="G40" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H40" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="47.25" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4377,22 +4377,22 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D41" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E41" s="17" t="str">
-        <x:v>Not supplied by this scan projection</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by this scan projection</x:v>
       </x:c>
       <x:c r="F41" s="17" t="str">
-        <x:v>NULL; gateway presence does not prove authentication type.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL; gateway presence does not prove authentication type.</x:v>
       </x:c>
       <x:c r="G41" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H41" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="47.25" customHeight="1">
       <x:c r="A42" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4403,22 +4403,22 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D42" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
-        <x:v>No verified credential identity in this input</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: No verified credential identity in this input</x:v>
       </x:c>
       <x:c r="F42" s="4" t="str">
-        <x:v>Unknown. Never infer Personal or Service Account from a hostname.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Unknown. Never infer Personal or Service Account from a hostname.</x:v>
       </x:c>
       <x:c r="G42" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H42" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="47.25" customHeight="1">
       <x:c r="A43" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -4429,22 +4429,22 @@
         <x:v>nvarchar(30)</x:v>
       </x:c>
       <x:c r="D43" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E43" s="17" t="str">
-        <x:v>Query evidence classification</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Query evidence classification</x:v>
       </x:c>
       <x:c r="F43" s="17" t="str">
-        <x:v>Partial when authentication or identity evidence is unavailable. Unknown is not a pass.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Partial when authentication or identity evidence is unavailable. Unknown is not a pass.</x:v>
       </x:c>
       <x:c r="G43" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H43" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="47.25" customHeight="1">
       <x:c r="A44" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -4455,22 +4455,22 @@
         <x:v>uniqueidentifier</x:v>
       </x:c>
       <x:c r="D44" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E44" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="F44" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="G44" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H44" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="47.25" customHeight="1">
       <x:c r="A45" s="17" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -4481,22 +4481,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D45" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E45" s="17" t="str">
-        <x:v>datasets[].id</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasets[].id</x:v>
       </x:c>
       <x:c r="F45" s="17" t="str">
-        <x:v>Only direct source-observed edges.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Only direct source-observed edges.</x:v>
       </x:c>
       <x:c r="G45" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="47.25" customHeight="1">
       <x:c r="A46" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -4507,22 +4507,22 @@
         <x:v>nvarchar(50)</x:v>
       </x:c>
       <x:c r="D46" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E46" s="4" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="F46" s="4" t="str">
-        <x:v>Dataset</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Dataset</x:v>
       </x:c>
       <x:c r="G46" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H46" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="47.25" customHeight="1">
       <x:c r="A47" s="17" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -4533,22 +4533,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D47" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E47" s="17" t="str">
-        <x:v>datasets[].datasourceUsages[].datasourceInstanceId joined to datasourceInstances[].datasourceId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasets[].datasourceUsages[].datasourceInstanceId joined to datasourceInstances[].datasourceId</x:v>
       </x:c>
       <x:c r="F47" s="17" t="str">
-        <x:v>Retain missing endpoints for review; never match by label.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Retain missing endpoints for review; never match by label.</x:v>
       </x:c>
       <x:c r="G47" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H47" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="47.25" customHeight="1">
       <x:c r="A48" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -4559,22 +4559,22 @@
         <x:v>nvarchar(30)</x:v>
       </x:c>
       <x:c r="D48" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E48" s="4" t="str">
-        <x:v>Join result</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Join result</x:v>
       </x:c>
       <x:c r="F48" s="4" t="str">
-        <x:v>Observed if both endpoints resolve; Unresolved otherwise.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Observed if both endpoints resolve; Unresolved otherwise.</x:v>
       </x:c>
       <x:c r="G48" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="47.25" customHeight="1">
       <x:c r="A49" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4585,22 +4585,22 @@
         <x:v>uniqueidentifier</x:v>
       </x:c>
       <x:c r="D49" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E49" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="F49" s="17" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="G49" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H49" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="47.25" customHeight="1">
       <x:c r="A50" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4611,22 +4611,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D50" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E50" s="4" t="str">
-        <x:v>reports[].id</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: reports[].id</x:v>
       </x:c>
       <x:c r="F50" s="4" t="str">
-        <x:v>Report ID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Report ID.</x:v>
       </x:c>
       <x:c r="G50" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H50" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="47.25" customHeight="1">
       <x:c r="A51" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4637,22 +4637,22 @@
         <x:v>nvarchar(50)</x:v>
       </x:c>
       <x:c r="D51" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E51" s="17" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="F51" s="17" t="str">
-        <x:v>Report</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Report</x:v>
       </x:c>
       <x:c r="G51" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H51" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="47.25" customHeight="1">
       <x:c r="A52" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4663,22 +4663,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D52" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E52" s="4" t="str">
-        <x:v>reports[].datasetId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: reports[].datasetId</x:v>
       </x:c>
       <x:c r="F52" s="4" t="str">
-        <x:v>Exact model ID; keep cross-workspace dependencies.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Exact model ID; keep cross-workspace dependencies.</x:v>
       </x:c>
       <x:c r="G52" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H52" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="47.25" customHeight="1">
       <x:c r="A53" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4689,22 +4689,22 @@
         <x:v>nvarchar(50)</x:v>
       </x:c>
       <x:c r="D53" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E53" s="17" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="F53" s="17" t="str">
-        <x:v>Dataset</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Dataset</x:v>
       </x:c>
       <x:c r="G53" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H53" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="47.25" customHeight="1">
       <x:c r="A54" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4715,22 +4715,22 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D54" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E54" s="4" t="str">
-        <x:v>Source relationship</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source relationship</x:v>
       </x:c>
       <x:c r="F54" s="4" t="str">
-        <x:v>UsesSemanticModel</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: UsesSemanticModel</x:v>
       </x:c>
       <x:c r="G54" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H54" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="47.25" customHeight="1">
       <x:c r="A55" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -4741,22 +4741,22 @@
         <x:v>nvarchar(30)</x:v>
       </x:c>
       <x:c r="D55" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E55" s="17" t="str">
-        <x:v>Endpoint resolution</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Endpoint resolution</x:v>
       </x:c>
       <x:c r="F55" s="17" t="str">
-        <x:v>Observed if model is in inventory; Unresolved otherwise.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Observed if model is in inventory; Unresolved otherwise.</x:v>
       </x:c>
       <x:c r="G55" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H55" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="47.25" customHeight="1">
       <x:c r="A56" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4767,22 +4767,22 @@
         <x:v>uniqueidentifier</x:v>
       </x:c>
       <x:c r="D56" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E56" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="F56" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="G56" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H56" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="47.25" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="58.5" customHeight="1">
       <x:c r="A57" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4793,22 +4793,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D57" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E57" s="17" t="str">
-        <x:v>artifact/workspace users[].graphId, otherwise explicit identifier</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: artifact/workspace users[].graphId, otherwise explicit identifier</x:v>
       </x:c>
       <x:c r="F57" s="17" t="str">
-        <x:v>Keep the V1 namespace: graphId uses PowerBIGraphID; fallback identifier uses PowerBIPrincipalIdentifier. Never use a display name. A later graphId requires continuity review, not silent rekeying.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Keep the V1 namespace: graphId uses PowerBIGraphID; fallback identifier uses PowerBIPrincipalIdentifier. Never use a display name. A later graphId requires continuity review, not silent rekeying.</x:v>
       </x:c>
       <x:c r="G57" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H57" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="47.25" customHeight="1">
       <x:c r="A58" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4819,22 +4819,22 @@
         <x:v>nvarchar(60)</x:v>
       </x:c>
       <x:c r="D58" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E58" s="4" t="str">
-        <x:v>Documented identifier source</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Documented identifier source</x:v>
       </x:c>
       <x:c r="F58" s="4" t="str">
-        <x:v>PowerBIGraphID for graphId; PowerBIPrincipalIdentifier for identifier fallback. Keep the namespace with its native key.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: PowerBIGraphID for graphId; PowerBIPrincipalIdentifier for identifier fallback. Keep the namespace with its native key.</x:v>
       </x:c>
       <x:c r="G58" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H58" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="47.25" customHeight="1">
       <x:c r="A59" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4845,22 +4845,22 @@
         <x:v>nvarchar(30)</x:v>
       </x:c>
       <x:c r="D59" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E59" s="17" t="str">
-        <x:v>users[].principalType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].principalType</x:v>
       </x:c>
       <x:c r="F59" s="17" t="str">
-        <x:v>User, Group, App, or None as supplied; never turn every principal into a person.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: User, Group, App, or None as supplied; never turn every principal into a person.</x:v>
       </x:c>
       <x:c r="G59" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H59" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="47.25" customHeight="1">
       <x:c r="A60" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4871,22 +4871,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D60" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E60" s="4" t="str">
-        <x:v>users[].displayName</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].displayName</x:v>
       </x:c>
       <x:c r="F60" s="4" t="str">
-        <x:v>Display only; optional.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Display only; optional.</x:v>
       </x:c>
       <x:c r="G60" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H60" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="47.25" customHeight="1">
       <x:c r="A61" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4897,22 +4897,22 @@
         <x:v>nvarchar(320)</x:v>
       </x:c>
       <x:c r="D61" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E61" s="17" t="str">
-        <x:v>users[].emailAddress</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].emailAddress</x:v>
       </x:c>
       <x:c r="F61" s="17" t="str">
-        <x:v>Preserve explicit email only; identifier or UPN is not an implicit fallback.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Preserve explicit email only; identifier or UPN is not an implicit fallback.</x:v>
       </x:c>
       <x:c r="G61" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H61" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="47.25" customHeight="1">
       <x:c r="A62" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -4923,19 +4923,19 @@
         <x:v>nvarchar(500)</x:v>
       </x:c>
       <x:c r="D62" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E62" s="4" t="str">
-        <x:v>Not supplied by scan principal fields</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by scan principal fields</x:v>
       </x:c>
       <x:c r="F62" s="4" t="str">
-        <x:v>NULL; access-right strings are roles, not enabled state.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL; access-right strings are roles, not enabled state.</x:v>
       </x:c>
       <x:c r="G62" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H62" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="36" customHeight="1">
@@ -5068,7 +5068,7 @@
         <x:v>https://learn.microsoft.com/en-us/graph/api/resources/user?view=graph-rest-1.0</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="36" customHeight="1">
+    <x:row r="68" ht="47.25" customHeight="1">
       <x:c r="A68" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5079,22 +5079,22 @@
         <x:v>uniqueidentifier</x:v>
       </x:c>
       <x:c r="D68" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E68" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="F68" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="G68" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H68" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="47.25" customHeight="1">
       <x:c r="A69" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5105,22 +5105,22 @@
         <x:v>nvarchar(50)</x:v>
       </x:c>
       <x:c r="D69" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E69" s="17" t="str">
-        <x:v>Parent source entity</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Parent source entity</x:v>
       </x:c>
       <x:c r="F69" s="17" t="str">
-        <x:v>Workspace / PersonalGroup / Project / Collection / Report / Dataset / Workbook / PublishedDatasource / Workflow; use the exact inventory namespace.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Workspace / PersonalGroup / Project / Collection / Report / Dataset / Workbook / PublishedDatasource / Workflow; use the exact inventory namespace.</x:v>
       </x:c>
       <x:c r="G69" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H69" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="47.25" customHeight="1">
       <x:c r="A70" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5131,22 +5131,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D70" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E70" s="4" t="str">
-        <x:v>Parent native object key</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Parent native object key</x:v>
       </x:c>
       <x:c r="F70" s="4" t="str">
-        <x:v>Use exact workspace or asset ID. Do not use the label.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Use exact workspace or asset ID. Do not use the label.</x:v>
       </x:c>
       <x:c r="G70" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H70" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="47.25" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="58.5" customHeight="1">
       <x:c r="A71" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5157,22 +5157,22 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D71" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E71" s="17" t="str">
-        <x:v>workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
       </x:c>
       <x:c r="F71" s="17" t="str">
-        <x:v>Access with native access-right fields; TechnicalOwner from reports.createdById, which Microsoft explicitly defines as report owner; ModifiedBy from reports.modifiedById. Neither assigns business ownership.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Access with native access-right fields; TechnicalOwner from reports.createdById, which Microsoft explicitly defines as report owner; ModifiedBy from reports.modifiedById. Neither assigns business ownership.</x:v>
       </x:c>
       <x:c r="G71" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H71" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="47.25" customHeight="1">
       <x:c r="A72" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5183,22 +5183,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D72" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E72" s="4" t="str">
-        <x:v>workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
       </x:c>
       <x:c r="F72" s="4" t="str">
-        <x:v>Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
       </x:c>
       <x:c r="G72" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H72" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="47.25" customHeight="1">
       <x:c r="A73" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5209,22 +5209,22 @@
         <x:v>nvarchar(60)</x:v>
       </x:c>
       <x:c r="D73" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E73" s="17" t="str">
-        <x:v>Documented reference kind</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Documented reference kind</x:v>
       </x:c>
       <x:c r="F73" s="17" t="str">
-        <x:v>PowerBIPrincipalIdentifier for raw identifier when present; otherwise PowerBIGraphID for graphId. Resolved account identity can use PowerBIGraphID independently.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: PowerBIPrincipalIdentifier for raw identifier when present; otherwise PowerBIGraphID for graphId. Resolved account identity can use PowerBIGraphID independently.</x:v>
       </x:c>
       <x:c r="G73" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H73" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="47.25" customHeight="1">
       <x:c r="A74" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5235,22 +5235,22 @@
         <x:v>nvarchar(200)</x:v>
       </x:c>
       <x:c r="D74" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E74" s="4" t="str">
-        <x:v>Verified reference-to-Platform_Users join</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Verified reference-to-Platform_Users join</x:v>
       </x:c>
       <x:c r="F74" s="4" t="str">
-        <x:v>Populate only after exact unique namespace match. NULL when unresolved; preserve raw source reference.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Populate only after exact unique namespace match. NULL when unresolved; preserve raw source reference.</x:v>
       </x:c>
       <x:c r="G74" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H74" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="47.25" customHeight="1">
       <x:c r="A75" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5261,22 +5261,22 @@
         <x:v>nvarchar(60)</x:v>
       </x:c>
       <x:c r="D75" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E75" s="17" t="str">
-        <x:v>Resolved Platform_Users.IdentifierNamespace</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Resolved Platform_Users.IdentifierNamespace</x:v>
       </x:c>
       <x:c r="F75" s="17" t="str">
-        <x:v>NULL when unresolved. Must accompany NativePrincipalID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL when unresolved. Must accompany NativePrincipalID.</x:v>
       </x:c>
       <x:c r="G75" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H75" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76" ht="36" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="47.25" customHeight="1">
       <x:c r="A76" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5287,22 +5287,22 @@
         <x:v>nvarchar(100)</x:v>
       </x:c>
       <x:c r="D76" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E76" s="4" t="str">
-        <x:v>Native access-right property when explicitly supplied</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Native access-right property when explicitly supplied</x:v>
       </x:c>
       <x:c r="F76" s="4" t="str">
-        <x:v>NULL for pure ownership/author relationships. Do not invent workspace privileges from Champion assignment.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL for pure ownership/author relationships. Do not invent workspace privileges from Champion assignment.</x:v>
       </x:c>
       <x:c r="G76" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H76" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="47.25" customHeight="1">
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="58.5" customHeight="1">
       <x:c r="A77" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -5313,25 +5313,25 @@
         <x:v>nvarchar(40)</x:v>
       </x:c>
       <x:c r="D77" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="E77" s="17" t="str">
-        <x:v>Reference resolution result</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Reference resolution result</x:v>
       </x:c>
       <x:c r="F77" s="17" t="str">
-        <x:v>ReadyForEmailMatch when the account and email resolve; MissingEmail, MissingSourceReference, UnresolvedUserReference, or UnverifiedMapping otherwise. This does not prove a directory match. Route unresolved cases to Platform Manager.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: ReadyForEmailMatch when the account and email resolve; MissingEmail, MissingSourceReference, UnresolvedUserReference, or UnverifiedMapping otherwise. This does not prove a directory match. Route unresolved cases to Platform Manager.</x:v>
       </x:c>
       <x:c r="G77" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H77" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R604359f482d34fa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74472e52ad94676"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5758,7 +5758,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H18" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="47.25" customHeight="1">
@@ -5775,7 +5775,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>AlteryxGallery.collections.CollectionId</x:v>
+        <x:v>ar_source.Alteryx_Collections.CollectionId (SQL adapter for AlteryxGallery.collections.CollectionId)</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
         <x:v>Preserve exact source text. Scope comes from Run_Context.</x:v>
@@ -5784,7 +5784,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H19" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="47.25" customHeight="1">
@@ -5810,7 +5810,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H20" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="47.25" customHeight="1">
@@ -5827,7 +5827,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
-        <x:v>AlteryxGallery.collections.Name</x:v>
+        <x:v>ar_source.Alteryx_Collections.Name (SQL adapter for AlteryxGallery.collections.Name)</x:v>
       </x:c>
       <x:c r="F21" s="17" t="str">
         <x:v>Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
@@ -5836,7 +5836,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="47.25" customHeight="1">
@@ -5862,7 +5862,7 @@
         <x:v>Always NULL in this profile; existence is not an explicit active status.</x:v>
       </x:c>
       <x:c r="H22" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="47.25" customHeight="1">
@@ -5888,7 +5888,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H23" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="47.25" customHeight="1">
@@ -5905,7 +5905,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>AlteryxGallery.appInfos._id</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.AppInfoId (SQL adapter for AlteryxGallery.appInfos._id)</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
         <x:v>Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
@@ -5914,7 +5914,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H24" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="47.25" customHeight="1">
@@ -5940,7 +5940,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H25" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="47.25" customHeight="1">
@@ -5957,7 +5957,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>One published Revisions entry, then one primary Applications entry: MetaInfo.Name</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.RevisionsJson -&gt; one published revision -&gt; one primary application -&gt; MetaInfo.Name (SQL adapter for One published Revisions entry, then one primary Applications entry: MetaInfo.Name)</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
         <x:v>If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
@@ -5966,7 +5966,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H26" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="47.25" customHeight="1">
@@ -5983,7 +5983,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E27" s="17" t="str">
-        <x:v>AlteryxGallery.appInfos.Revisions[].RevisionId where IsPublishedRevision=true</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.RevisionsJson -&gt; one published revision RevisionId (SQL adapter for AlteryxGallery.appInfos.Revisions[].RevisionId where IsPublishedRevision=true)</x:v>
       </x:c>
       <x:c r="F27" s="17" t="str">
         <x:v>Exactly one published revision required. Multiple or no candidates route to Platform Manager; never choose max revision silently.</x:v>
@@ -5992,7 +5992,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="47.25" customHeight="1">
@@ -6009,7 +6009,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
-        <x:v>AlteryxGallery.appInfos.IsDeleted</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.IsDeleted (SQL adapter for AlteryxGallery.appInfos.IsDeleted)</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
         <x:v>Explicit true maps to Deleted, false maps to Present. Missing stays NULL. Neither value proves business retirement.</x:v>
@@ -6018,7 +6018,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H28" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="47.25" customHeight="1">
@@ -6044,7 +6044,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="47.25" customHeight="1">
@@ -6061,7 +6061,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
-        <x:v>AlteryxGallery.collections.CollectionId</x:v>
+        <x:v>ar_source.Alteryx_Collections.CollectionId (SQL adapter for AlteryxGallery.collections.CollectionId)</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
         <x:v>Resolve exact ID in this delivery scope.</x:v>
@@ -6070,7 +6070,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H30" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="47.25" customHeight="1">
@@ -6087,7 +6087,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>AlteryxGallery.collections.Apps[].ApplicationId</x:v>
+        <x:v>ar_source.Alteryx_Collections.AppsJson -&gt; Apps[].ApplicationId (SQL adapter for AlteryxGallery.collections.Apps[].ApplicationId)</x:v>
       </x:c>
       <x:c r="F31" s="17" t="str">
         <x:v>Preserve unmatched IDs as unresolved relationships.</x:v>
@@ -6096,7 +6096,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="47.25" customHeight="1">
@@ -6122,7 +6122,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H32" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="47.25" customHeight="1">
@@ -6148,7 +6148,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="47.25" customHeight="1">
@@ -6174,7 +6174,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H34" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="47.25" customHeight="1">
@@ -6200,7 +6200,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="47.25" customHeight="1">
@@ -6226,7 +6226,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H36" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="47.25" customHeight="1">
@@ -6252,7 +6252,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="47.25" customHeight="1">
@@ -6278,7 +6278,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H38" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="47.25" customHeight="1">
@@ -6304,7 +6304,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H39" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="47.25" customHeight="1">
@@ -6330,7 +6330,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H40" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="47.25" customHeight="1">
@@ -6356,7 +6356,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H41" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="47.25" customHeight="1">
@@ -6382,7 +6382,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H42" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="47.25" customHeight="1">
@@ -6408,7 +6408,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H43" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="47.25" customHeight="1">
@@ -6434,7 +6434,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H44" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="47.25" customHeight="1">
@@ -6460,7 +6460,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="47.25" customHeight="1">
@@ -6486,7 +6486,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H46" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="47.25" customHeight="1">
@@ -6512,7 +6512,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H47" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="47.25" customHeight="1">
@@ -6538,7 +6538,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="47.25" customHeight="1">
@@ -6564,7 +6564,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H49" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="47.25" customHeight="1">
@@ -6590,7 +6590,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H50" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="47.25" customHeight="1">
@@ -6616,7 +6616,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H51" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="47.25" customHeight="1">
@@ -6642,7 +6642,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H52" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="47.25" customHeight="1">
@@ -6668,7 +6668,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H53" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="47.25" customHeight="1">
@@ -6694,7 +6694,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H54" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="47.25" customHeight="1">
@@ -6720,7 +6720,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="H55" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="47.25" customHeight="1">
@@ -6746,7 +6746,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H56" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="47.25" customHeight="1">
@@ -6763,7 +6763,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E57" s="17" t="str">
-        <x:v>AlteryxGallery.users._id</x:v>
+        <x:v>ar_source.Alteryx_Users.UserId (SQL adapter for AlteryxGallery.users._id)</x:v>
       </x:c>
       <x:c r="F57" s="17" t="str">
         <x:v>Exact Mongo ID text; Windows SID is a different namespace.</x:v>
@@ -6772,7 +6772,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H57" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="47.25" customHeight="1">
@@ -6798,7 +6798,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H58" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="47.25" customHeight="1">
@@ -6824,7 +6824,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H59" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="47.25" customHeight="1">
@@ -6841,7 +6841,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E60" s="4" t="str">
-        <x:v>AlteryxGallery.users.FirstName + LastName</x:v>
+        <x:v>ar_source.Alteryx_Users.FirstName + LastName (SQL adapter for AlteryxGallery.users.FirstName + LastName)</x:v>
       </x:c>
       <x:c r="F60" s="4" t="str">
         <x:v>Join available name parts for display only.</x:v>
@@ -6850,7 +6850,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H60" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="47.25" customHeight="1">
@@ -6867,7 +6867,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E61" s="17" t="str">
-        <x:v>AlteryxGallery.users.Email</x:v>
+        <x:v>ar_source.Alteryx_Users.Email (SQL adapter for AlteryxGallery.users.Email)</x:v>
       </x:c>
       <x:c r="F61" s="17" t="str">
         <x:v>Preserve explicit email; WindowsIdentity.Name is not a fallback.</x:v>
@@ -6876,7 +6876,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H61" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="47.25" customHeight="1">
@@ -6893,7 +6893,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E62" s="4" t="str">
-        <x:v>AlteryxGallery.users.Active</x:v>
+        <x:v>ar_source.Alteryx_Users.Active (SQL adapter for AlteryxGallery.users.Active)</x:v>
       </x:c>
       <x:c r="F62" s="4" t="str">
         <x:v>Explicit native boolean as text, NULL if missing. Native status is not Entra accountEnabled.</x:v>
@@ -6902,7 +6902,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H62" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="36" customHeight="1">
@@ -7058,7 +7058,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H68" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="47.25" customHeight="1">
@@ -7084,7 +7084,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H69" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="47.25" customHeight="1">
@@ -7110,10 +7110,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H70" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="47.25" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="58.5" customHeight="1">
       <x:c r="A71" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -7127,7 +7127,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="E71" s="17" t="str">
-        <x:v>collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping</x:v>
+        <x:v>ar_source.Alteryx_Collections.OwnerId / UsersJson -&gt; Users[].UserId; ar_source.Alteryx_AppInfos.CreatedBy (SQL adapter for collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping)</x:v>
       </x:c>
       <x:c r="F71" s="17" t="str">
         <x:v>TechnicalOwner for collection OwnerId; CollectionMember for Users; CreatedBy for appInfos.CreatedBy. Current workflow TechnicalOwner is unverified</x:v>
@@ -7136,10 +7136,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H71" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="47.25" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="58.5" customHeight="1">
       <x:c r="A72" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -7153,7 +7153,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E72" s="4" t="str">
-        <x:v>collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping</x:v>
+        <x:v>ar_source.Alteryx_Collections.OwnerId / UsersJson -&gt; Users[].UserId; ar_source.Alteryx_AppInfos.CreatedBy (SQL adapter for collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping)</x:v>
       </x:c>
       <x:c r="F72" s="4" t="str">
         <x:v>Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
@@ -7162,7 +7162,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H72" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="47.25" customHeight="1">
@@ -7188,7 +7188,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H73" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="47.25" customHeight="1">
@@ -7214,7 +7214,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H74" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="47.25" customHeight="1">
@@ -7240,7 +7240,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H75" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="47.25" customHeight="1">
@@ -7266,7 +7266,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="H76" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="47.25" customHeight="1">
@@ -7292,13 +7292,13 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="H77" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64f4e2b5f72b477e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfecaf919c8f4108"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8697,7 +8697,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H42" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="I42" s="4" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -8706,7 +8706,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K42" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="36" customHeight="1">
@@ -8776,7 +8776,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K44" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="36" customHeight="1">
@@ -8802,16 +8802,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
-        <x:v>workspaces[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceId. Existing scan export: workspaces[].id</x:v>
       </x:c>
       <x:c r="I45" s="17" t="str">
-        <x:v>Preserve exact source text. Scope comes from Run_Context.</x:v>
+        <x:v>Fabric inventory: Preserve the native workspace ID as text. Existing scan export: Preserve exact source text. Scope comes from Run_Context.</x:v>
       </x:c>
       <x:c r="J45" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K45" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="36" customHeight="1">
@@ -8872,7 +8872,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H47" s="17" t="str">
-        <x:v>AlteryxGallery.collections.CollectionId</x:v>
+        <x:v>ar_source.Alteryx_Collections.CollectionId (SQL adapter for AlteryxGallery.collections.CollectionId)</x:v>
       </x:c>
       <x:c r="I47" s="17" t="str">
         <x:v>Preserve exact source text. Scope comes from Run_Context.</x:v>
@@ -8881,7 +8881,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K47" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="36" customHeight="1">
@@ -8907,16 +8907,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
-        <x:v>Source entity kind</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceType. Existing scan export: Source entity kind</x:v>
       </x:c>
       <x:c r="I48" s="4" t="str">
-        <x:v>Use workspaces[].type, commonly Workspace or PersonalGroup.</x:v>
+        <x:v>Fabric inventory: Use the validated native type. Missing type stops extraction. Existing scan export: Use workspaces[].type, commonly Workspace or PersonalGroup.</x:v>
       </x:c>
       <x:c r="J48" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K48" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="36" customHeight="1">
@@ -8986,10 +8986,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K50" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="47.25" customHeight="1">
       <x:c r="A51" s="17" t="str">
         <x:v>Workspaces</x:v>
       </x:c>
@@ -9012,16 +9012,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H51" s="17" t="str">
-        <x:v>workspaces[].name</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceName. Existing scan export: workspaces[].name</x:v>
       </x:c>
       <x:c r="I51" s="17" t="str">
-        <x:v>Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
+        <x:v>Fabric inventory: Use the observed name; never use it as a key. Existing scan export: Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
       </x:c>
       <x:c r="J51" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K51" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="36" customHeight="1">
@@ -9082,7 +9082,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H53" s="17" t="str">
-        <x:v>AlteryxGallery.collections.Name</x:v>
+        <x:v>ar_source.Alteryx_Collections.Name (SQL adapter for AlteryxGallery.collections.Name)</x:v>
       </x:c>
       <x:c r="I53" s="17" t="str">
         <x:v>Current technical name only. A rename updates this attribute without changing registry identity.</x:v>
@@ -9091,7 +9091,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K53" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="36" customHeight="1">
@@ -9114,19 +9114,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G54" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H54" s="4" t="str">
-        <x:v>workspaces[].state</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: workspaces[].state</x:v>
       </x:c>
       <x:c r="I54" s="4" t="str">
-        <x:v>Preserve the native state; never infer account status.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Preserve the native state; never infer account status.</x:v>
       </x:c>
       <x:c r="J54" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K54" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="36" customHeight="1">
@@ -9196,7 +9196,7 @@
         <x:v>Always NULL in this profile; existence is not an explicit active status.</x:v>
       </x:c>
       <x:c r="K56" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="36" customHeight="1">
@@ -9222,7 +9222,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H57" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="I57" s="17" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -9231,7 +9231,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K57" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="36" customHeight="1">
@@ -9301,10 +9301,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K59" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="47.25" customHeight="1">
       <x:c r="A60" s="4" t="str">
         <x:v>Assets</x:v>
       </x:c>
@@ -9327,16 +9327,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H60" s="4" t="str">
-        <x:v>workspaces[].reports[].id or datasets[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemId. Existing scan export: workspaces[].reports[].id or datasets[].id</x:v>
       </x:c>
       <x:c r="I60" s="4" t="str">
-        <x:v>Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
+        <x:v>Fabric inventory: Preserve the native item ID as text. Existing scan export: Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
       </x:c>
       <x:c r="J60" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K60" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="36" customHeight="1">
@@ -9397,7 +9397,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H62" s="4" t="str">
-        <x:v>AlteryxGallery.appInfos._id</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.AppInfoId (SQL adapter for AlteryxGallery.appInfos._id)</x:v>
       </x:c>
       <x:c r="I62" s="4" t="str">
         <x:v>Preserve exact ID. Mongo Extended JSON $oid is decoded to its exact text; do not use filename or revision ID.</x:v>
@@ -9406,7 +9406,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K62" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="36" customHeight="1">
@@ -9432,16 +9432,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H63" s="17" t="str">
-        <x:v>Source object namespace</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemType. Existing scan export: Source object namespace</x:v>
       </x:c>
       <x:c r="I63" s="17" t="str">
-        <x:v>Report or Dataset, matching the source array.</x:v>
+        <x:v>Fabric inventory: Report stays Report. SemanticModel, Semantic model, and Dataset map to Dataset. Existing scan export: Report or Dataset, matching the source array.</x:v>
       </x:c>
       <x:c r="J63" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K63" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="36" customHeight="1">
@@ -9511,10 +9511,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K65" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="47.25" customHeight="1">
       <x:c r="A66" s="4" t="str">
         <x:v>Assets</x:v>
       </x:c>
@@ -9537,16 +9537,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H66" s="4" t="str">
-        <x:v>reports[].name or datasets[].name</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemName. Existing scan export: reports[].name or datasets[].name</x:v>
       </x:c>
       <x:c r="I66" s="4" t="str">
-        <x:v>If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
+        <x:v>Fabric inventory: Use the observed item name. Existing scan export: If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
       </x:c>
       <x:c r="J66" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K66" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="36" customHeight="1">
@@ -9584,7 +9584,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="47.25" customHeight="1">
+    <x:row r="68" ht="58.5" customHeight="1">
       <x:c r="A68" s="4" t="str">
         <x:v>Assets</x:v>
       </x:c>
@@ -9607,7 +9607,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H68" s="4" t="str">
-        <x:v>One published Revisions entry, then one primary Applications entry: MetaInfo.Name</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.RevisionsJson -&gt; one published revision -&gt; one primary application -&gt; MetaInfo.Name (SQL adapter for One published Revisions entry, then one primary Applications entry: MetaInfo.Name)</x:v>
       </x:c>
       <x:c r="I68" s="4" t="str">
         <x:v>If ambiguous or absent, retain raw evidence and route to Platform Manager. Never invent a name to pass validation.</x:v>
@@ -9616,7 +9616,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K68" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="47.25" customHeight="1">
@@ -9639,19 +9639,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G69" s="17" t="str">
-        <x:v>Leave NULL</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H69" s="17" t="str">
-        <x:v>No native revision in the baseline scan fields</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: No native revision in the baseline scan fields</x:v>
       </x:c>
       <x:c r="I69" s="17" t="str">
-        <x:v>Do not synthesize a version from modified time.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Do not synthesize a version from modified time.</x:v>
       </x:c>
       <x:c r="J69" s="17" t="str">
-        <x:v>Always NULL for baseline scan projection.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: Always NULL for baseline scan projection.</x:v>
       </x:c>
       <x:c r="K69" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="47.25" customHeight="1">
@@ -9712,7 +9712,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H71" s="17" t="str">
-        <x:v>AlteryxGallery.appInfos.Revisions[].RevisionId where IsPublishedRevision=true</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.RevisionsJson -&gt; one published revision RevisionId (SQL adapter for AlteryxGallery.appInfos.Revisions[].RevisionId where IsPublishedRevision=true)</x:v>
       </x:c>
       <x:c r="I71" s="17" t="str">
         <x:v>Exactly one published revision required. Multiple or no candidates route to Platform Manager; never choose max revision silently.</x:v>
@@ -9721,7 +9721,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K71" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="36" customHeight="1">
@@ -9744,19 +9744,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G72" s="4" t="str">
-        <x:v>Leave NULL</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H72" s="4" t="str">
-        <x:v>Not projected by baseline inventory</x:v>
+        <x:v>Fabric inventory: unavailable. Existing scan export: Not projected by baseline inventory</x:v>
       </x:c>
       <x:c r="I72" s="4" t="str">
-        <x:v>Inventory presence is recorded by the observation itself.</x:v>
+        <x:v>Fabric inventory: leave NULL; this source does not establish the value. Existing scan export: Inventory presence is recorded by the observation itself.</x:v>
       </x:c>
       <x:c r="J72" s="4" t="str">
-        <x:v>Always NULL unless an authoritative lifecycle field is separately approved.</x:v>
+        <x:v>Fabric inventory: always NULL. Existing scan export: Always NULL unless an authoritative lifecycle field is separately approved.</x:v>
       </x:c>
       <x:c r="K72" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="36" customHeight="1">
@@ -9817,7 +9817,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H74" s="4" t="str">
-        <x:v>AlteryxGallery.appInfos.IsDeleted</x:v>
+        <x:v>ar_source.Alteryx_AppInfos.IsDeleted (SQL adapter for AlteryxGallery.appInfos.IsDeleted)</x:v>
       </x:c>
       <x:c r="I74" s="4" t="str">
         <x:v>Explicit true maps to Deleted, false maps to Present. Missing stays NULL. Neither value proves business retirement.</x:v>
@@ -9826,7 +9826,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K74" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="36" customHeight="1">
@@ -9852,7 +9852,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H75" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Both profiles: existing immutable delivery manifest</x:v>
       </x:c>
       <x:c r="I75" s="17" t="str">
         <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
@@ -9861,7 +9861,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K75" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="36" customHeight="1">
@@ -9931,7 +9931,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K77" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="36" customHeight="1">
@@ -9957,16 +9957,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H78" s="4" t="str">
-        <x:v>Parent workspaces[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.WorkspaceId. Existing scan export: Parent workspaces[].id</x:v>
       </x:c>
       <x:c r="I78" s="4" t="str">
-        <x:v>Resolve exact ID in this delivery scope.</x:v>
+        <x:v>Fabric inventory: Preserve the native workspace ID. Existing scan export: Resolve exact ID in this delivery scope.</x:v>
       </x:c>
       <x:c r="J78" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K78" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="36" customHeight="1">
@@ -10027,7 +10027,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H80" s="4" t="str">
-        <x:v>AlteryxGallery.collections.CollectionId</x:v>
+        <x:v>ar_source.Alteryx_Collections.CollectionId (SQL adapter for AlteryxGallery.collections.CollectionId)</x:v>
       </x:c>
       <x:c r="I80" s="4" t="str">
         <x:v>Resolve exact ID in this delivery scope.</x:v>
@@ -10036,7 +10036,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K80" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="36" customHeight="1">
@@ -10062,16 +10062,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H81" s="17" t="str">
-        <x:v>Nested reports[].id / datasets[].id</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemId. Existing scan export: Nested reports[].id / datasets[].id</x:v>
       </x:c>
       <x:c r="I81" s="17" t="str">
-        <x:v>Preserve unmatched IDs as unresolved relationships.</x:v>
+        <x:v>Fabric inventory: Preserve the native item ID. Existing scan export: Preserve unmatched IDs as unresolved relationships.</x:v>
       </x:c>
       <x:c r="J81" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K81" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="36" customHeight="1">
@@ -10132,7 +10132,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H83" s="17" t="str">
-        <x:v>AlteryxGallery.collections.Apps[].ApplicationId</x:v>
+        <x:v>ar_source.Alteryx_Collections.AppsJson -&gt; Apps[].ApplicationId (SQL adapter for AlteryxGallery.collections.Apps[].ApplicationId)</x:v>
       </x:c>
       <x:c r="I83" s="17" t="str">
         <x:v>Preserve unmatched IDs as unresolved relationships.</x:v>
@@ -10141,7 +10141,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K83" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="36" customHeight="1">
@@ -10167,16 +10167,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H84" s="4" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: registry_source.FabricInventory.ItemType. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="I84" s="4" t="str">
-        <x:v>Report / Dataset</x:v>
+        <x:v>Fabric inventory: Use Report or Dataset with the same type mapping as Assets. Existing scan export: Report / Dataset</x:v>
       </x:c>
       <x:c r="J84" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K84" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="36" customHeight="1">
@@ -10246,7 +10246,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K86" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="47.25" customHeight="1">
@@ -10272,16 +10272,16 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H87" s="17" t="str">
-        <x:v>Query relationship label</x:v>
+        <x:v>Fabric inventory: Direct source containment (query constant). Existing scan export: Query relationship label</x:v>
       </x:c>
       <x:c r="I87" s="17" t="str">
-        <x:v>ContainedIn; observed membership never assigns business ownership.</x:v>
+        <x:v>Fabric inventory: Use ContainedIn. This is membership, not lineage. Existing scan export: ContainedIn; observed membership never assigns business ownership.</x:v>
       </x:c>
       <x:c r="J87" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K87" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="47.25" customHeight="1">
@@ -10351,10 +10351,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K89" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="47.25" customHeight="1">
       <x:c r="A90" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10374,19 +10374,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G90" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H90" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="I90" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="J90" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K90" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="36" customHeight="1">
@@ -10456,7 +10456,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K92" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="47.25" customHeight="1">
@@ -10479,19 +10479,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G93" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H93" s="17" t="str">
-        <x:v>datasourceInstances[].datasourceId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceId</x:v>
       </x:c>
       <x:c r="I93" s="17" t="str">
-        <x:v>Exact native datasource ID. Do not hash connection secrets or invent a name-based ID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Exact native datasource ID. Do not hash connection secrets or invent a name-based ID.</x:v>
       </x:c>
       <x:c r="J93" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K93" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="47.25" customHeight="1">
@@ -10561,7 +10561,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K95" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="47.25" customHeight="1">
@@ -10584,19 +10584,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G96" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H96" s="4" t="str">
-        <x:v>datasourceInstances[].datasourceType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceType</x:v>
       </x:c>
       <x:c r="I96" s="4" t="str">
-        <x:v>Optional readable technical label. No business meaning is inferred.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Optional readable technical label. No business meaning is inferred.</x:v>
       </x:c>
       <x:c r="J96" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K96" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="47.25" customHeight="1">
@@ -10666,7 +10666,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K98" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="47.25" customHeight="1">
@@ -10689,19 +10689,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G99" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H99" s="17" t="str">
-        <x:v>datasourceInstances[].datasourceType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].datasourceType</x:v>
       </x:c>
       <x:c r="I99" s="17" t="str">
-        <x:v>Map Oracle to Oracle, Sql to SQL Server; preserve other known types. Undefined only when technology is unavailable.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Map Oracle to Oracle, Sql to SQL Server; preserve other known types. Undefined only when technology is unavailable.</x:v>
       </x:c>
       <x:c r="J99" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K99" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="47.25" customHeight="1">
@@ -10771,7 +10771,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K101" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="47.25" customHeight="1">
@@ -10794,19 +10794,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G102" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H102" s="4" t="str">
-        <x:v>Not supplied by scan datasource instance</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by scan datasource instance</x:v>
       </x:c>
       <x:c r="I102" s="4" t="str">
-        <x:v>NULL. Report/model storage mode must not be inferred from datasource type.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL. Report/model storage mode must not be inferred from datasource type.</x:v>
       </x:c>
       <x:c r="J102" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K102" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="47.25" customHeight="1">
@@ -10876,10 +10876,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K104" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="47.25" customHeight="1">
       <x:c r="A105" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10899,19 +10899,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G105" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H105" s="17" t="str">
-        <x:v>datasourceInstances[].connectionDetails.server</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].connectionDetails.server</x:v>
       </x:c>
       <x:c r="I105" s="17" t="str">
-        <x:v>Sanitized host only. No URL tokens or credentials.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Sanitized host only. No URL tokens or credentials.</x:v>
       </x:c>
       <x:c r="J105" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K105" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="36" customHeight="1">
@@ -10981,10 +10981,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K107" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="47.25" customHeight="1">
       <x:c r="A108" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11004,19 +11004,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G108" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H108" s="4" t="str">
-        <x:v>datasourceInstances[].connectionDetails.database</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasourceInstances[].connectionDetails.database</x:v>
       </x:c>
       <x:c r="I108" s="4" t="str">
-        <x:v>Database name when present.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Database name when present.</x:v>
       </x:c>
       <x:c r="J108" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K108" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="36" customHeight="1">
@@ -11086,7 +11086,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K110" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="47.25" customHeight="1">
@@ -11109,19 +11109,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G111" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H111" s="17" t="str">
-        <x:v>Not supplied by this scan projection</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by this scan projection</x:v>
       </x:c>
       <x:c r="I111" s="17" t="str">
-        <x:v>NULL; gateway presence does not prove authentication type.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL; gateway presence does not prove authentication type.</x:v>
       </x:c>
       <x:c r="J111" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K111" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="47.25" customHeight="1">
@@ -11191,7 +11191,7 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K113" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="47.25" customHeight="1">
@@ -11214,19 +11214,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G114" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H114" s="4" t="str">
-        <x:v>No verified credential identity in this input</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: No verified credential identity in this input</x:v>
       </x:c>
       <x:c r="I114" s="4" t="str">
-        <x:v>Unknown. Never infer Personal or Service Account from a hostname.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Unknown. Never infer Personal or Service Account from a hostname.</x:v>
       </x:c>
       <x:c r="J114" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K114" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="47.25" customHeight="1">
@@ -11296,10 +11296,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K116" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="47.25" customHeight="1">
       <x:c r="A117" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11319,19 +11319,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G117" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H117" s="17" t="str">
-        <x:v>Query evidence classification</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Query evidence classification</x:v>
       </x:c>
       <x:c r="I117" s="17" t="str">
-        <x:v>Partial when authentication or identity evidence is unavailable. Unknown is not a pass.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Partial when authentication or identity evidence is unavailable. Unknown is not a pass.</x:v>
       </x:c>
       <x:c r="J117" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K117" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="36" customHeight="1">
@@ -11401,10 +11401,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K119" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="120" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="47.25" customHeight="1">
       <x:c r="A120" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -11424,19 +11424,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G120" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H120" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="I120" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="J120" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K120" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="36" customHeight="1">
@@ -11506,10 +11506,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K122" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="47.25" customHeight="1">
       <x:c r="A123" s="17" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -11529,19 +11529,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G123" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H123" s="17" t="str">
-        <x:v>datasets[].id</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasets[].id</x:v>
       </x:c>
       <x:c r="I123" s="17" t="str">
-        <x:v>Only direct source-observed edges.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Only direct source-observed edges.</x:v>
       </x:c>
       <x:c r="J123" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K123" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="36" customHeight="1">
@@ -11611,10 +11611,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K125" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="47.25" customHeight="1">
       <x:c r="A126" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -11634,19 +11634,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G126" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H126" s="4" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="I126" s="4" t="str">
-        <x:v>Dataset</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Dataset</x:v>
       </x:c>
       <x:c r="J126" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K126" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="36" customHeight="1">
@@ -11716,10 +11716,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K128" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="129" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="47.25" customHeight="1">
       <x:c r="A129" s="17" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -11739,19 +11739,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G129" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H129" s="17" t="str">
-        <x:v>datasets[].datasourceUsages[].datasourceInstanceId joined to datasourceInstances[].datasourceId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: datasets[].datasourceUsages[].datasourceInstanceId joined to datasourceInstances[].datasourceId</x:v>
       </x:c>
       <x:c r="I129" s="17" t="str">
-        <x:v>Retain missing endpoints for review; never match by label.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Retain missing endpoints for review; never match by label.</x:v>
       </x:c>
       <x:c r="J129" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K129" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="36" customHeight="1">
@@ -11821,10 +11821,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K131" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="132" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="47.25" customHeight="1">
       <x:c r="A132" s="4" t="str">
         <x:v>Asset_Connections</x:v>
       </x:c>
@@ -11844,19 +11844,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G132" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H132" s="4" t="str">
-        <x:v>Join result</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Join result</x:v>
       </x:c>
       <x:c r="I132" s="4" t="str">
-        <x:v>Observed if both endpoints resolve; Unresolved otherwise.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Observed if both endpoints resolve; Unresolved otherwise.</x:v>
       </x:c>
       <x:c r="J132" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K132" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="36" customHeight="1">
@@ -11926,10 +11926,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K134" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="135" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="47.25" customHeight="1">
       <x:c r="A135" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -11949,19 +11949,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G135" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H135" s="17" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="I135" s="17" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="J135" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K135" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="36" customHeight="1">
@@ -12031,10 +12031,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K137" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="138" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="47.25" customHeight="1">
       <x:c r="A138" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12054,19 +12054,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G138" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H138" s="4" t="str">
-        <x:v>reports[].id</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: reports[].id</x:v>
       </x:c>
       <x:c r="I138" s="4" t="str">
-        <x:v>Report ID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Report ID.</x:v>
       </x:c>
       <x:c r="J138" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K138" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="36" customHeight="1">
@@ -12136,10 +12136,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K140" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="141" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="47.25" customHeight="1">
       <x:c r="A141" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12159,19 +12159,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G141" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H141" s="17" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="I141" s="17" t="str">
-        <x:v>Report</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Report</x:v>
       </x:c>
       <x:c r="J141" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K141" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="36" customHeight="1">
@@ -12241,10 +12241,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K143" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="144" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="47.25" customHeight="1">
       <x:c r="A144" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12264,19 +12264,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G144" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H144" s="4" t="str">
-        <x:v>reports[].datasetId</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: reports[].datasetId</x:v>
       </x:c>
       <x:c r="I144" s="4" t="str">
-        <x:v>Exact model ID; keep cross-workspace dependencies.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Exact model ID; keep cross-workspace dependencies.</x:v>
       </x:c>
       <x:c r="J144" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K144" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="36" customHeight="1">
@@ -12346,10 +12346,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K146" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="147" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="47.25" customHeight="1">
       <x:c r="A147" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12369,19 +12369,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G147" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H147" s="17" t="str">
-        <x:v>Source branch</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source branch</x:v>
       </x:c>
       <x:c r="I147" s="17" t="str">
-        <x:v>Dataset</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Dataset</x:v>
       </x:c>
       <x:c r="J147" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K147" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="36" customHeight="1">
@@ -12451,10 +12451,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K149" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="150" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="47.25" customHeight="1">
       <x:c r="A150" s="4" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12474,19 +12474,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G150" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H150" s="4" t="str">
-        <x:v>Source relationship</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Source relationship</x:v>
       </x:c>
       <x:c r="I150" s="4" t="str">
-        <x:v>UsesSemanticModel</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: UsesSemanticModel</x:v>
       </x:c>
       <x:c r="J150" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K150" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="36" customHeight="1">
@@ -12556,10 +12556,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K152" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="153" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="47.25" customHeight="1">
       <x:c r="A153" s="17" t="str">
         <x:v>Asset_Dependencies</x:v>
       </x:c>
@@ -12579,19 +12579,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G153" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H153" s="17" t="str">
-        <x:v>Endpoint resolution</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Endpoint resolution</x:v>
       </x:c>
       <x:c r="I153" s="17" t="str">
-        <x:v>Observed if model is in inventory; Unresolved otherwise.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Observed if model is in inventory; Unresolved otherwise.</x:v>
       </x:c>
       <x:c r="J153" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K153" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="36" customHeight="1">
@@ -12661,10 +12661,10 @@
         <x:v>Emit no rows for an uncollected dataset. Set CoverageStatus=NotCollected; do not create NULL placeholder records.</x:v>
       </x:c>
       <x:c r="K155" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="156" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="47.25" customHeight="1">
       <x:c r="A156" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -12684,19 +12684,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G156" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H156" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="I156" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="J156" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K156" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="36" customHeight="1">
@@ -12766,10 +12766,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K158" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159" ht="47.25" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="58.5" customHeight="1">
       <x:c r="A159" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -12789,19 +12789,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G159" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H159" s="17" t="str">
-        <x:v>artifact/workspace users[].graphId, otherwise explicit identifier</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: artifact/workspace users[].graphId, otherwise explicit identifier</x:v>
       </x:c>
       <x:c r="I159" s="17" t="str">
-        <x:v>Keep the V1 namespace: graphId uses PowerBIGraphID; fallback identifier uses PowerBIPrincipalIdentifier. Never use a display name. A later graphId requires continuity review, not silent rekeying.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Keep the V1 namespace: graphId uses PowerBIGraphID; fallback identifier uses PowerBIPrincipalIdentifier. Never use a display name. A later graphId requires continuity review, not silent rekeying.</x:v>
       </x:c>
       <x:c r="J159" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K159" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="36" customHeight="1">
@@ -12862,7 +12862,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H161" s="17" t="str">
-        <x:v>AlteryxGallery.users._id</x:v>
+        <x:v>ar_source.Alteryx_Users.UserId (SQL adapter for AlteryxGallery.users._id)</x:v>
       </x:c>
       <x:c r="I161" s="17" t="str">
         <x:v>Exact Mongo ID text; Windows SID is a different namespace.</x:v>
@@ -12871,10 +12871,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K161" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="47.25" customHeight="1">
       <x:c r="A162" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -12894,19 +12894,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G162" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H162" s="4" t="str">
-        <x:v>Documented identifier source</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Documented identifier source</x:v>
       </x:c>
       <x:c r="I162" s="4" t="str">
-        <x:v>PowerBIGraphID for graphId; PowerBIPrincipalIdentifier for identifier fallback. Keep the namespace with its native key.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: PowerBIGraphID for graphId; PowerBIPrincipalIdentifier for identifier fallback. Keep the namespace with its native key.</x:v>
       </x:c>
       <x:c r="J162" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K162" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="36" customHeight="1">
@@ -12976,10 +12976,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K164" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="165" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="47.25" customHeight="1">
       <x:c r="A165" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -12999,19 +12999,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G165" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H165" s="17" t="str">
-        <x:v>users[].principalType</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].principalType</x:v>
       </x:c>
       <x:c r="I165" s="17" t="str">
-        <x:v>User, Group, App, or None as supplied; never turn every principal into a person.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: User, Group, App, or None as supplied; never turn every principal into a person.</x:v>
       </x:c>
       <x:c r="J165" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K165" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="36" customHeight="1">
@@ -13081,10 +13081,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K167" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="168" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="47.25" customHeight="1">
       <x:c r="A168" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -13104,19 +13104,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G168" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H168" s="4" t="str">
-        <x:v>users[].displayName</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].displayName</x:v>
       </x:c>
       <x:c r="I168" s="4" t="str">
-        <x:v>Display only; optional.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Display only; optional.</x:v>
       </x:c>
       <x:c r="J168" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K168" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="36" customHeight="1">
@@ -13177,7 +13177,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H170" s="4" t="str">
-        <x:v>AlteryxGallery.users.FirstName + LastName</x:v>
+        <x:v>ar_source.Alteryx_Users.FirstName + LastName (SQL adapter for AlteryxGallery.users.FirstName + LastName)</x:v>
       </x:c>
       <x:c r="I170" s="4" t="str">
         <x:v>Join available name parts for display only.</x:v>
@@ -13186,10 +13186,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K170" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="171" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="47.25" customHeight="1">
       <x:c r="A171" s="17" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -13209,19 +13209,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G171" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H171" s="17" t="str">
-        <x:v>users[].emailAddress</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: users[].emailAddress</x:v>
       </x:c>
       <x:c r="I171" s="17" t="str">
-        <x:v>Preserve explicit email only; identifier or UPN is not an implicit fallback.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Preserve explicit email only; identifier or UPN is not an implicit fallback.</x:v>
       </x:c>
       <x:c r="J171" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K171" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="36" customHeight="1">
@@ -13282,7 +13282,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H173" s="17" t="str">
-        <x:v>AlteryxGallery.users.Email</x:v>
+        <x:v>ar_source.Alteryx_Users.Email (SQL adapter for AlteryxGallery.users.Email)</x:v>
       </x:c>
       <x:c r="I173" s="17" t="str">
         <x:v>Preserve explicit email; WindowsIdentity.Name is not a fallback.</x:v>
@@ -13291,10 +13291,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K173" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="174" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="47.25" customHeight="1">
       <x:c r="A174" s="4" t="str">
         <x:v>Platform_Users</x:v>
       </x:c>
@@ -13314,19 +13314,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G174" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H174" s="4" t="str">
-        <x:v>Not supplied by scan principal fields</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Not supplied by scan principal fields</x:v>
       </x:c>
       <x:c r="I174" s="4" t="str">
-        <x:v>NULL; access-right strings are roles, not enabled state.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL; access-right strings are roles, not enabled state.</x:v>
       </x:c>
       <x:c r="J174" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K174" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="36" customHeight="1">
@@ -13387,7 +13387,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H176" s="4" t="str">
-        <x:v>AlteryxGallery.users.Active</x:v>
+        <x:v>ar_source.Alteryx_Users.Active (SQL adapter for AlteryxGallery.users.Active)</x:v>
       </x:c>
       <x:c r="I176" s="4" t="str">
         <x:v>Explicit native boolean as text, NULL if missing. Native status is not Entra accountEnabled.</x:v>
@@ -13396,7 +13396,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K176" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="36" customHeight="1">
@@ -13924,7 +13924,7 @@
         <x:v>https://learn.microsoft.com/en-us/graph/api/resources/user?view=graph-rest-1.0</x:v>
       </x:c>
     </x:row>
-    <x:row r="192" ht="36" customHeight="1">
+    <x:row r="192" ht="47.25" customHeight="1">
       <x:c r="A192" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -13944,19 +13944,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G192" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H192" s="4" t="str">
-        <x:v>Existing delivery manifest</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Existing delivery manifest</x:v>
       </x:c>
       <x:c r="I192" s="4" t="str">
-        <x:v>Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Repeat the same delivery UUID on its dataset rows. A retry uses this UUID only for identical immutable input. A later delivery uses a new UUID.</x:v>
       </x:c>
       <x:c r="J192" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K192" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="36" customHeight="1">
@@ -14026,10 +14026,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K194" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="195" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="47.25" customHeight="1">
       <x:c r="A195" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14049,19 +14049,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G195" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H195" s="17" t="str">
-        <x:v>Parent source entity</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Parent source entity</x:v>
       </x:c>
       <x:c r="I195" s="17" t="str">
-        <x:v>Workspace / PersonalGroup / Project / Collection / Report / Dataset / Workbook / PublishedDatasource / Workflow; use the exact inventory namespace.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Workspace / PersonalGroup / Project / Collection / Report / Dataset / Workbook / PublishedDatasource / Workflow; use the exact inventory namespace.</x:v>
       </x:c>
       <x:c r="J195" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K195" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="36" customHeight="1">
@@ -14131,10 +14131,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K197" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="198" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="47.25" customHeight="1">
       <x:c r="A198" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14154,19 +14154,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G198" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H198" s="4" t="str">
-        <x:v>Parent native object key</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Parent native object key</x:v>
       </x:c>
       <x:c r="I198" s="4" t="str">
-        <x:v>Use exact workspace or asset ID. Do not use the label.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Use exact workspace or asset ID. Do not use the label.</x:v>
       </x:c>
       <x:c r="J198" s="4" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K198" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="36" customHeight="1">
@@ -14236,10 +14236,10 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K200" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="201" ht="47.25" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="58.5" customHeight="1">
       <x:c r="A201" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14259,19 +14259,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G201" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H201" s="17" t="str">
-        <x:v>workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
       </x:c>
       <x:c r="I201" s="17" t="str">
-        <x:v>Access with native access-right fields; TechnicalOwner from reports.createdById, which Microsoft explicitly defines as report owner; ModifiedBy from reports.modifiedById. Neither assigns business ownership.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Access with native access-right fields; TechnicalOwner from reports.createdById, which Microsoft explicitly defines as report owner; ModifiedBy from reports.modifiedById. Neither assigns business ownership.</x:v>
       </x:c>
       <x:c r="J201" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K201" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="47.25" customHeight="1">
@@ -14309,7 +14309,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="203" ht="47.25" customHeight="1">
+    <x:row r="203" ht="58.5" customHeight="1">
       <x:c r="A203" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14332,7 +14332,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="H203" s="17" t="str">
-        <x:v>collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping</x:v>
+        <x:v>ar_source.Alteryx_Collections.OwnerId / UsersJson -&gt; Users[].UserId; ar_source.Alteryx_AppInfos.CreatedBy (SQL adapter for collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping)</x:v>
       </x:c>
       <x:c r="I203" s="17" t="str">
         <x:v>TechnicalOwner for collection OwnerId; CollectionMember for Users; CreatedBy for appInfos.CreatedBy. Current workflow TechnicalOwner is unverified</x:v>
@@ -14341,7 +14341,7 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K203" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="47.25" customHeight="1">
@@ -14364,19 +14364,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G204" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H204" s="4" t="str">
-        <x:v>workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: workspaces[].users[] and datasets[].users[] / reports[].users[]</x:v>
       </x:c>
       <x:c r="I204" s="4" t="str">
-        <x:v>Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
       </x:c>
       <x:c r="J204" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K204" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="47.25" customHeight="1">
@@ -14414,7 +14414,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="206" ht="47.25" customHeight="1">
+    <x:row r="206" ht="58.5" customHeight="1">
       <x:c r="A206" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14437,7 +14437,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H206" s="4" t="str">
-        <x:v>collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping</x:v>
+        <x:v>ar_source.Alteryx_Collections.OwnerId / UsersJson -&gt; Users[].UserId; ar_source.Alteryx_AppInfos.CreatedBy (SQL adapter for collections.OwnerId, collections.Users[].UserId, appInfos.CreatedBy; optional verified current owner mapping)</x:v>
       </x:c>
       <x:c r="I206" s="4" t="str">
         <x:v>Preserve the raw reference when supplied. NULL for missing reference or unverified workflow ownership; retain the object-role row for Platform Manager.</x:v>
@@ -14446,7 +14446,7 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K206" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="47.25" customHeight="1">
@@ -14469,19 +14469,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G207" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H207" s="17" t="str">
-        <x:v>Documented reference kind</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Documented reference kind</x:v>
       </x:c>
       <x:c r="I207" s="17" t="str">
-        <x:v>PowerBIPrincipalIdentifier for raw identifier when present; otherwise PowerBIGraphID for graphId. Resolved account identity can use PowerBIGraphID independently.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: PowerBIPrincipalIdentifier for raw identifier when present; otherwise PowerBIGraphID for graphId. Resolved account identity can use PowerBIGraphID independently.</x:v>
       </x:c>
       <x:c r="J207" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K207" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="47.25" customHeight="1">
@@ -14551,10 +14551,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K209" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="210" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="47.25" customHeight="1">
       <x:c r="A210" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14574,19 +14574,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G210" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H210" s="4" t="str">
-        <x:v>Verified reference-to-Platform_Users join</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Verified reference-to-Platform_Users join</x:v>
       </x:c>
       <x:c r="I210" s="4" t="str">
-        <x:v>Populate only after exact unique namespace match. NULL when unresolved; preserve raw source reference.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: Populate only after exact unique namespace match. NULL when unresolved; preserve raw source reference.</x:v>
       </x:c>
       <x:c r="J210" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K210" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="36" customHeight="1">
@@ -14656,10 +14656,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K212" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="213" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="47.25" customHeight="1">
       <x:c r="A213" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14679,19 +14679,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G213" s="17" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H213" s="17" t="str">
-        <x:v>Resolved Platform_Users.IdentifierNamespace</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Resolved Platform_Users.IdentifierNamespace</x:v>
       </x:c>
       <x:c r="I213" s="17" t="str">
-        <x:v>NULL when unresolved. Must accompany NativePrincipalID.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL when unresolved. Must accompany NativePrincipalID.</x:v>
       </x:c>
       <x:c r="J213" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K213" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="36" customHeight="1">
@@ -14761,10 +14761,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K215" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="216" ht="36" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="47.25" customHeight="1">
       <x:c r="A216" s="4" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14784,19 +14784,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G216" s="4" t="str">
-        <x:v>Conditional</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H216" s="4" t="str">
-        <x:v>Native access-right property when explicitly supplied</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Native access-right property when explicitly supplied</x:v>
       </x:c>
       <x:c r="I216" s="4" t="str">
-        <x:v>NULL for pure ownership/author relationships. Do not invent workspace privileges from Champion assignment.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: NULL for pure ownership/author relationships. Do not invent workspace privileges from Champion assignment.</x:v>
       </x:c>
       <x:c r="J216" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K216" s="4" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="36" customHeight="1">
@@ -14866,10 +14866,10 @@
         <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
       </x:c>
       <x:c r="K218" s="4" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="219" ht="47.25" customHeight="1">
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="58.5" customHeight="1">
       <x:c r="A219" s="17" t="str">
         <x:v>Object_Users</x:v>
       </x:c>
@@ -14889,19 +14889,19 @@
         <x:v>PowerBI</x:v>
       </x:c>
       <x:c r="G219" s="17" t="str">
-        <x:v>Required</x:v>
+        <x:v>Profile dependent</x:v>
       </x:c>
       <x:c r="H219" s="17" t="str">
-        <x:v>Reference resolution result</x:v>
+        <x:v>Fabric inventory: not collected. Existing scan export: Reference resolution result</x:v>
       </x:c>
       <x:c r="I219" s="17" t="str">
-        <x:v>ReadyForEmailMatch when the account and email resolve; MissingEmail, MissingSourceReference, UnresolvedUserReference, or UnverifiedMapping otherwise. This does not prove a directory match. Route unresolved cases to Platform Manager.</x:v>
+        <x:v>Fabric inventory: emit no rows; record NotCollected coverage. Existing scan export: ReadyForEmailMatch when the account and email resolve; MissingEmail, MissingSourceReference, UnresolvedUserReference, or UnverifiedMapping otherwise. This does not prove a directory match. Route unresolved cases to Platform Manager.</x:v>
       </x:c>
       <x:c r="J219" s="17" t="str">
-        <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
+        <x:v>Fabric inventory: use headers only, without placeholder rows. Existing scan export: Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K219" s="17" t="str">
-        <x:v>https://learn.microsoft.com/en-us/rest/api/power-bi/admin/workspace-info-get-scan-result</x:v>
+        <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="47.25" customHeight="1">
@@ -14971,13 +14971,13 @@
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
       </x:c>
       <x:c r="K221" s="17" t="str">
-        <x:v>https://help.alteryx.com/current/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
+        <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07e1cb7fe20458f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43cdb629fb8b4ec6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17037,7 +17037,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R051096f7230a4476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8817cb2ed65d4e28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17138,7 +17138,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bf046ffe6d64350"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3746545f64e64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17203,7 +17203,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9741b60238184177"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62ab524e8fe4b35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17277,7 +17277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc4f8bf8eeb4745"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcd376d7e9549ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17360,7 +17360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20cec2209b044578"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79abd5f8fde34660"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17434,7 +17434,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1edf7f975e44418"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f2201369cc244a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17553,7 +17553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re13abeddd9eb4047"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eddcdc3d1d845b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Package V1.2 documentation, verification, and release artifacts
</commit_message>
<xml_diff>
--- a/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
+++ b/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R35e06569631d4547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R02d97914bffd4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="Rdfd902765592404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R306371199fef4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ff78ae54c4147ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R746ebc82870e40ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R695faf2619634fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="R4a4d6630eb8a4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="R32fc44687fd641ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R2794a9d89628442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="Re0c316331b194d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R21201718dbd34235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="Re1dc4cb9718f44d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R02803f40f78248bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R27ef375b836d411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Re42b7c9b960043d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="Raa76edd8102b4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R706ca3e3cead41ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R28034bfd27a34b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="R518a544153a94679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R280a5550c7354108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7c779a88de96474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R98609a8e68a54661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R10e17fd14ff94057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="Rf8ac10d2bd6e4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="Rcf5163258ade4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R02c2dc5c4b084c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="R9e0d9ade00a84c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R597e2a774d2e4fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="R648dd15adf76471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R1ea91791cd074426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R8c03e708b9bb4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Rae4e244ce4c74961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="R8a8e4ff0505f4409"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -758,7 +758,7 @@
         <x:v>2. Declare coverage</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Provide one Coverage row for each dataset in the agreed scope. Distinguish Complete, Partial, NotCollected, and Failed. Empty input does not prove absence.</x:v>
+        <x:v>Provide one Coverage row per dataset. Complete and Partial require exact delivered row counts. Failed and NotCollected require NULL counts and no data rows. Empty input does not prove absence.</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>Coverage</x:v>
@@ -777,15 +777,15 @@
       </x:c>
       <x:c r="D10" s="4" t="str"/>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+    <x:row r="11" ht="47.25" customHeight="1">
       <x:c r="A11" s="17" t="str">
-        <x:v>4. Validate and load</x:v>
+        <x:v>4. Validate and accept</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>Ignore only fully blank template rows. Quarantine invalid nonblank rows. Validate keys, references, and coverage before manual SQL Server staging.</x:v>
+        <x:v>Stage all nonblank records for validation. Structural errors block the whole delivery. The registry operator accepts valid deliveries, including Partial coverage and unresolved references. Assign unresolved cases to Platform Manager; preserve original evidence dates.</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Platform Manager</x:v>
+        <x:v>Registry operator</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str"/>
     </x:row>
@@ -806,7 +806,7 @@
         <x:v>Refresh identity</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Resolve native objects within PlatformCode, PlatformInstanceKey, NativeScopeKey, native object type, and native ID. Names remain display fields.</x:v>
+        <x:v>Resolve objects by platform, instance, native scope, entity kind, and native ID. Asset identity also includes native asset type. Workspace subtype, names, and email do not identify an object.</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Registry reconciliation</x:v>
@@ -946,7 +946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37cb9a51087c417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954f0b7a33f440d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1020,7 +1020,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re348627782404da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae71ea844534097"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1112,7 +1112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref01c47526934f4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ca802527de84404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1204,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7a5777105a948f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a006110e91f4a54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1278,7 +1278,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169aecea494e415e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R433f4badf717405f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1397,7 +1397,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbccb69c61b1c4f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe42702ea1b2426a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1775,7 +1775,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -1792,10 +1792,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -2312,7 +2312,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="F37" s="17" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="G37" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -3364,7 +3364,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e780e0296d4a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40c4eaf2650b48f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3742,7 +3742,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -3759,10 +3759,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -5331,7 +5331,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74472e52ad94676"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dcfee9fb89f486d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5709,7 +5709,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -5726,10 +5726,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -7298,7 +7298,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfecaf919c8f4108"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd10b1c7670438b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8569,7 +8569,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="47.25" customHeight="1">
+    <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8583,7 +8583,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F39" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -8595,16 +8595,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I39" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J39" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K39" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="47.25" customHeight="1">
+    <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="4" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8618,7 +8618,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -8630,16 +8630,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I40" s="4" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J40" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K40" s="4" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="47.25" customHeight="1">
+    <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8653,7 +8653,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E41" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F41" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -8665,10 +8665,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I41" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J41" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K41" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -10459,7 +10459,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="47.25" customHeight="1">
+    <x:row r="93" ht="58.5" customHeight="1">
       <x:c r="A93" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10473,7 +10473,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E93" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F93" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10494,7 +10494,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="47.25" customHeight="1">
+    <x:row r="94" ht="58.5" customHeight="1">
       <x:c r="A94" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10508,7 +10508,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E94" s="4" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F94" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10529,7 +10529,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="47.25" customHeight="1">
+    <x:row r="95" ht="58.5" customHeight="1">
       <x:c r="A95" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10543,7 +10543,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E95" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F95" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10578,7 +10578,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E96" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F96" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10613,7 +10613,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E97" s="17" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F97" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10648,7 +10648,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E98" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F98" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10669,7 +10669,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="47.25" customHeight="1">
+    <x:row r="99" ht="58.5" customHeight="1">
       <x:c r="A99" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10683,7 +10683,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E99" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F99" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10704,7 +10704,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="47.25" customHeight="1">
+    <x:row r="100" ht="58.5" customHeight="1">
       <x:c r="A100" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10718,7 +10718,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E100" s="4" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F100" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="I100" s="4" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="J100" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -10739,7 +10739,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="47.25" customHeight="1">
+    <x:row r="101" ht="58.5" customHeight="1">
       <x:c r="A101" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10753,7 +10753,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E101" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F101" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10774,7 +10774,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="47.25" customHeight="1">
+    <x:row r="102" ht="58.5" customHeight="1">
       <x:c r="A102" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10788,7 +10788,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E102" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F102" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10809,7 +10809,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="47.25" customHeight="1">
+    <x:row r="103" ht="58.5" customHeight="1">
       <x:c r="A103" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10823,7 +10823,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E103" s="17" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F103" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10844,7 +10844,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="47.25" customHeight="1">
+    <x:row r="104" ht="58.5" customHeight="1">
       <x:c r="A104" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10858,7 +10858,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E104" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F104" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10893,7 +10893,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E105" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F105" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10914,7 +10914,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="36" customHeight="1">
+    <x:row r="106" ht="47.25" customHeight="1">
       <x:c r="A106" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10928,7 +10928,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E106" s="4" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F106" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10963,7 +10963,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E107" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F107" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10998,7 +10998,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E108" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F108" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11019,7 +11019,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="36" customHeight="1">
+    <x:row r="109" ht="47.25" customHeight="1">
       <x:c r="A109" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11033,7 +11033,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E109" s="17" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F109" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11068,7 +11068,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E110" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F110" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11103,7 +11103,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E111" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F111" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11138,7 +11138,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E112" s="4" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F112" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11173,7 +11173,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E113" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F113" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -11208,7 +11208,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E114" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F114" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11243,7 +11243,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E115" s="17" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F115" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11278,7 +11278,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E116" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F116" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11299,7 +11299,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="117" ht="47.25" customHeight="1">
+    <x:row r="117" ht="58.5" customHeight="1">
       <x:c r="A117" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11313,7 +11313,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E117" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F117" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11334,7 +11334,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="118" ht="36" customHeight="1">
+    <x:row r="118" ht="58.5" customHeight="1">
       <x:c r="A118" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11348,7 +11348,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E118" s="4" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F118" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11369,7 +11369,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="119" ht="47.25" customHeight="1">
+    <x:row r="119" ht="58.5" customHeight="1">
       <x:c r="A119" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11383,7 +11383,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E119" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F119" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -14977,7 +14977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43cdb629fb8b4ec6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra61eb6225581410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17037,7 +17037,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8817cb2ed65d4e28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25994da914184e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17138,7 +17138,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3746545f64e64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd747f99e6db44827"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17203,7 +17203,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62ab524e8fe4b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3812b6e9e2dd4ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17277,7 +17277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcd376d7e9549ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0a230eabe98481d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17360,7 +17360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79abd5f8fde34660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07e43b6624348aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17434,7 +17434,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f2201369cc244a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3daffe014da44b38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17553,7 +17553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eddcdc3d1d845b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c208403f7ee4d58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Analytic Registry V1.2 prototype (#1)
Ship reviewed application workflows, Excel contract, platform query pack, diagrams, and documentation. Preserve platform identity and business metadata boundaries. Verify portable archives and coherent artifact hashes.
</commit_message>
<xml_diff>
--- a/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
+++ b/analytic-registry/public/resources/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R35e06569631d4547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R02d97914bffd4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="Rdfd902765592404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R306371199fef4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ff78ae54c4147ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R746ebc82870e40ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R695faf2619634fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="R4a4d6630eb8a4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="R32fc44687fd641ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R2794a9d89628442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="Re0c316331b194d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R21201718dbd34235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="Re1dc4cb9718f44d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R02803f40f78248bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R27ef375b836d411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Re42b7c9b960043d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="Raa76edd8102b4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R706ca3e3cead41ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R28034bfd27a34b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="R518a544153a94679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R280a5550c7354108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7c779a88de96474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R98609a8e68a54661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R10e17fd14ff94057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="Rf8ac10d2bd6e4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="Rcf5163258ade4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R02c2dc5c4b084c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="R9e0d9ade00a84c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R597e2a774d2e4fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="R648dd15adf76471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R1ea91791cd074426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R8c03e708b9bb4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Rae4e244ce4c74961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="R8a8e4ff0505f4409"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -758,7 +758,7 @@
         <x:v>2. Declare coverage</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Provide one Coverage row for each dataset in the agreed scope. Distinguish Complete, Partial, NotCollected, and Failed. Empty input does not prove absence.</x:v>
+        <x:v>Provide one Coverage row per dataset. Complete and Partial require exact delivered row counts. Failed and NotCollected require NULL counts and no data rows. Empty input does not prove absence.</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>Coverage</x:v>
@@ -777,15 +777,15 @@
       </x:c>
       <x:c r="D10" s="4" t="str"/>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+    <x:row r="11" ht="47.25" customHeight="1">
       <x:c r="A11" s="17" t="str">
-        <x:v>4. Validate and load</x:v>
+        <x:v>4. Validate and accept</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>Ignore only fully blank template rows. Quarantine invalid nonblank rows. Validate keys, references, and coverage before manual SQL Server staging.</x:v>
+        <x:v>Stage all nonblank records for validation. Structural errors block the whole delivery. The registry operator accepts valid deliveries, including Partial coverage and unresolved references. Assign unresolved cases to Platform Manager; preserve original evidence dates.</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Platform Manager</x:v>
+        <x:v>Registry operator</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str"/>
     </x:row>
@@ -806,7 +806,7 @@
         <x:v>Refresh identity</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Resolve native objects within PlatformCode, PlatformInstanceKey, NativeScopeKey, native object type, and native ID. Names remain display fields.</x:v>
+        <x:v>Resolve objects by platform, instance, native scope, entity kind, and native ID. Asset identity also includes native asset type. Workspace subtype, names, and email do not identify an object.</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Registry reconciliation</x:v>
@@ -946,7 +946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37cb9a51087c417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954f0b7a33f440d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1020,7 +1020,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re348627782404da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae71ea844534097"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1112,7 +1112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref01c47526934f4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ca802527de84404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1204,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7a5777105a948f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a006110e91f4a54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1278,7 +1278,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169aecea494e415e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R433f4badf717405f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1397,7 +1397,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbccb69c61b1c4f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe42702ea1b2426a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1775,7 +1775,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -1792,10 +1792,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -2312,7 +2312,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="F37" s="17" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="G37" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -3364,7 +3364,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e780e0296d4a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40c4eaf2650b48f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3742,7 +3742,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -3759,10 +3759,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -5331,7 +5331,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74472e52ad94676"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dcfee9fb89f486d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5709,7 +5709,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -5726,10 +5726,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -7298,7 +7298,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfecaf919c8f4108"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd10b1c7670438b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8569,7 +8569,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="47.25" customHeight="1">
+    <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8583,7 +8583,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F39" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -8595,16 +8595,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I39" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J39" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K39" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="47.25" customHeight="1">
+    <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="4" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8618,7 +8618,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -8630,16 +8630,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I40" s="4" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J40" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K40" s="4" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="47.25" customHeight="1">
+    <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8653,7 +8653,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E41" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F41" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -8665,10 +8665,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I41" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J41" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K41" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -10459,7 +10459,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="47.25" customHeight="1">
+    <x:row r="93" ht="58.5" customHeight="1">
       <x:c r="A93" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10473,7 +10473,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E93" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F93" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10494,7 +10494,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="47.25" customHeight="1">
+    <x:row r="94" ht="58.5" customHeight="1">
       <x:c r="A94" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10508,7 +10508,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E94" s="4" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F94" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10529,7 +10529,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="47.25" customHeight="1">
+    <x:row r="95" ht="58.5" customHeight="1">
       <x:c r="A95" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10543,7 +10543,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E95" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F95" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10578,7 +10578,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E96" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F96" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10613,7 +10613,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E97" s="17" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F97" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10648,7 +10648,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E98" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F98" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10669,7 +10669,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="47.25" customHeight="1">
+    <x:row r="99" ht="58.5" customHeight="1">
       <x:c r="A99" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10683,7 +10683,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E99" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F99" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10704,7 +10704,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="47.25" customHeight="1">
+    <x:row r="100" ht="58.5" customHeight="1">
       <x:c r="A100" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10718,7 +10718,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E100" s="4" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F100" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="I100" s="4" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="J100" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -10739,7 +10739,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="47.25" customHeight="1">
+    <x:row r="101" ht="58.5" customHeight="1">
       <x:c r="A101" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10753,7 +10753,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E101" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F101" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10774,7 +10774,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="47.25" customHeight="1">
+    <x:row r="102" ht="58.5" customHeight="1">
       <x:c r="A102" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10788,7 +10788,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E102" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F102" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10809,7 +10809,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="47.25" customHeight="1">
+    <x:row r="103" ht="58.5" customHeight="1">
       <x:c r="A103" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10823,7 +10823,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E103" s="17" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F103" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10844,7 +10844,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="47.25" customHeight="1">
+    <x:row r="104" ht="58.5" customHeight="1">
       <x:c r="A104" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10858,7 +10858,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E104" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F104" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10893,7 +10893,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E105" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F105" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10914,7 +10914,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="36" customHeight="1">
+    <x:row r="106" ht="47.25" customHeight="1">
       <x:c r="A106" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10928,7 +10928,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E106" s="4" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F106" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10963,7 +10963,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E107" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F107" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10998,7 +10998,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E108" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F108" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11019,7 +11019,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="36" customHeight="1">
+    <x:row r="109" ht="47.25" customHeight="1">
       <x:c r="A109" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11033,7 +11033,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E109" s="17" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F109" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11068,7 +11068,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E110" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F110" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11103,7 +11103,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E111" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F111" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11138,7 +11138,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E112" s="4" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F112" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11173,7 +11173,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E113" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F113" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -11208,7 +11208,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E114" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F114" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11243,7 +11243,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E115" s="17" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F115" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11278,7 +11278,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E116" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F116" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11299,7 +11299,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="117" ht="47.25" customHeight="1">
+    <x:row r="117" ht="58.5" customHeight="1">
       <x:c r="A117" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11313,7 +11313,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E117" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F117" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11334,7 +11334,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="118" ht="36" customHeight="1">
+    <x:row r="118" ht="58.5" customHeight="1">
       <x:c r="A118" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11348,7 +11348,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E118" s="4" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F118" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11369,7 +11369,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="119" ht="47.25" customHeight="1">
+    <x:row r="119" ht="58.5" customHeight="1">
       <x:c r="A119" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11383,7 +11383,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E119" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F119" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -14977,7 +14977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43cdb629fb8b4ec6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra61eb6225581410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17037,7 +17037,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8817cb2ed65d4e28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25994da914184e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17138,7 +17138,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3746545f64e64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd747f99e6db44827"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17203,7 +17203,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62ab524e8fe4b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3812b6e9e2dd4ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17277,7 +17277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcd376d7e9549ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0a230eabe98481d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17360,7 +17360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79abd5f8fde34660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07e43b6624348aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17434,7 +17434,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f2201369cc244a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3daffe014da44b38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17553,7 +17553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eddcdc3d1d845b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c208403f7ee4d58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>